<commit_message>
Resolve open decisions, add /session-end skill, ship resource hub v1
Confirms name (final), grade range, and cost (free); leaves Showcase
format open. Adds a per-week resource hub scaffold: Chart/Chord
Chart/Reference Track URL columns on the song library, joined to the
schedule by a new Song Title column, rendered as a Resources column
on both the Schedule and Song Library tables (falls back to "Coming
soon" until a leader fills in a URL). Also adds the /session-end
skill this workflow itself uses.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/Worship Music School - Rollout Schedule.xlsx
+++ b/deliverables/Worship Music School - Rollout Schedule.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Rollout Schedule" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Rollout Schedule'!$A$3:$H$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Rollout Schedule'!$A$3:$I$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,17 +51,12 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <i val="1"/>
       <color rgb="00999999"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -76,11 +71,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FBF3E9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4A6"/>
       </patternFill>
     </fill>
     <fill>
@@ -120,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -136,18 +126,15 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -515,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -580,6 +567,11 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
+          <t>Song Title</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
           <t>Milestones / Notes</t>
         </is>
       </c>
@@ -620,7 +612,12 @@
           <t>10,000 Reasons — introduce &amp; jam</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>10,000 Reasons (Bless the Lord)</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>LAUNCH NIGHT. Names, instruments, expectations, fun.</t>
         </is>
@@ -662,7 +659,12 @@
           <t>10,000 Reasons — learn &amp; play</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>10,000 Reasons (Bless the Lord)</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -700,7 +702,12 @@
           <t>What A Beautiful Name — begin</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>What A Beautiful Name</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -738,7 +745,12 @@
           <t>What A Beautiful Name — finish</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>What A Beautiful Name</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>MILESTONE: first song, start to finish.</t>
         </is>
@@ -780,7 +792,12 @@
           <t>This Is Amazing Grace — begin</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr"/>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>This Is Amazing Grace</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -818,7 +835,12 @@
           <t>This Is Amazing Grace — finish (to a click)</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr"/>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>This Is Amazing Grace</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -856,7 +878,12 @@
           <t>Build My Life — begin</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr"/>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Build My Life</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -894,7 +921,12 @@
           <t>Build My Life — finish (from a chart)</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr"/>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Build My Life</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -934,6 +966,11 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
+          <t>Stand By Me</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
           <t>Feel &amp; pocket; the famous bass line.</t>
         </is>
       </c>
@@ -974,7 +1011,12 @@
           <t>Goodness of God — begin (6/8 feel)</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Goodness of God</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1012,37 +1054,43 @@
           <t>Goodness of God — finish</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr"/>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Goodness of God</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Sun Nov 22</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Fall</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>— Thanksgiving break —</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr"/>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>— no meeting —</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr"/>
-      <c r="H15" s="8" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr"/>
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>Break — no meeting.</t>
         </is>
@@ -1086,6 +1134,11 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
+          <t>Joy to the World (Unspeakable Joy); Silent Night</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
           <t>Start Showcase prep.</t>
         </is>
       </c>
@@ -1126,7 +1179,12 @@
           <t>Christmas set: add O Come All Ye Faithful; polish</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr"/>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Joy to the World (Unspeakable Joy); Silent Night; O Come All Ye Faithful (Faithful)</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1164,401 +1222,448 @@
           <t>SHOWCASE — perform the Christmas set</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Joy to the World (Unspeakable Joy); Silent Night; O Come All Ye Faithful (Faithful)</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>MILESTONE: Fall Showcase. Invite parents/church.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Sun Dec 20</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>— Christmas break —</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr"/>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr"/>
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>— no meeting —</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr"/>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr"/>
+      <c r="H19" s="7" t="inlineStr"/>
+      <c r="I19" s="7" t="inlineStr">
         <is>
           <t>Break — no meeting.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Sun Dec 27</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>— Christmas break —</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr"/>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr"/>
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>— no meeting —</t>
         </is>
       </c>
-      <c r="G20" s="8" t="inlineStr"/>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr"/>
+      <c r="H20" s="7" t="inlineStr"/>
+      <c r="I20" s="7" t="inlineStr">
         <is>
           <t>Break — no meeting.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Sun Jan 3</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Winter</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Reset: the worshiping life</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E21" s="9" t="inlineStr">
         <is>
           <t>Colossians 3:1–17</t>
         </is>
       </c>
-      <c r="F21" s="10" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>Gear deep-dive I — strings &amp; keys, pedals</t>
         </is>
       </c>
-      <c r="G21" s="10" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t>Living Hope — begin</t>
         </is>
       </c>
-      <c r="H21" s="10" t="inlineStr">
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>Living Hope</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
         <is>
           <t>New term. Set individual goals.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>Sun Jan 10</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Winter</t>
         </is>
       </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>The full range of worship</t>
         </is>
       </c>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="E22" s="9" t="inlineStr">
         <is>
           <t>Psalm 13; Psalm 150</t>
         </is>
       </c>
-      <c r="F22" s="10" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Gear deep-dive II — drums &amp; vocals</t>
         </is>
       </c>
-      <c r="G22" s="10" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr">
         <is>
           <t>Living Hope — finish</t>
         </is>
       </c>
-      <c r="H22" s="10" t="inlineStr"/>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>Living Hope</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>Sun Jan 17</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>Winter</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>Young and setting the example</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t>1 Timothy 4:12</t>
         </is>
       </c>
-      <c r="F23" s="10" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>Communication &amp; tools (Planning Center)</t>
         </is>
       </c>
-      <c r="G23" s="10" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
         <is>
           <t>Graves Into Gardens — begin</t>
         </is>
       </c>
-      <c r="H23" s="10" t="inlineStr"/>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>Graves Into Gardens</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>Sun Jan 24</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>Winter</t>
         </is>
       </c>
-      <c r="D24" s="10" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>One body, many parts</t>
         </is>
       </c>
-      <c r="E24" s="10" t="inlineStr">
+      <c r="E24" s="9" t="inlineStr">
         <is>
           <t>1 Corinthians 12:12–27</t>
         </is>
       </c>
-      <c r="F24" s="10" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>Being a bandmate — rhythm-section lock</t>
         </is>
       </c>
-      <c r="G24" s="10" t="inlineStr">
+      <c r="G24" s="9" t="inlineStr">
         <is>
           <t>Isn't She Lovely — secular groove</t>
         </is>
       </c>
-      <c r="H24" s="10" t="inlineStr">
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>Isn't She Lovely</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="inlineStr">
         <is>
           <t>Rhythm section feature.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Sun Jan 31</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>Winter</t>
         </is>
       </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="D25" s="9" t="inlineStr">
         <is>
           <t>Chasing God's presence</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E25" s="9" t="inlineStr">
         <is>
           <t>Exodus 33:12–23; Psalm 84</t>
         </is>
       </c>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>Leading vs. playing</t>
         </is>
       </c>
-      <c r="G25" s="10" t="inlineStr">
+      <c r="G25" s="9" t="inlineStr">
         <is>
           <t>King of Kings — begin (a student leads)</t>
         </is>
       </c>
-      <c r="H25" s="10" t="inlineStr"/>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>King of Kings</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="B26" s="9" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Sun Feb 7</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>Winter</t>
         </is>
       </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="D26" s="9" t="inlineStr">
         <is>
           <t>Use what you've been given</t>
         </is>
       </c>
-      <c r="E26" s="10" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t>Matthew 25:14–30; 1 Peter 4:10–11</t>
         </is>
       </c>
-      <c r="F26" s="10" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>Building &amp; running a full set</t>
         </is>
       </c>
-      <c r="G26" s="10" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr">
         <is>
           <t>Assemble a full Winter set (3–4 songs)</t>
         </is>
       </c>
-      <c r="H26" s="10" t="inlineStr"/>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>Living Hope; Graves Into Gardens; Isn't She Lovely; King of Kings</t>
+        </is>
+      </c>
+      <c r="I26" s="9" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Sun Feb 14</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>Winter</t>
         </is>
       </c>
-      <c r="D27" s="10" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>Worship as witness</t>
         </is>
       </c>
-      <c r="E27" s="10" t="inlineStr">
+      <c r="E27" s="9" t="inlineStr">
         <is>
           <t>Psalm 40:1–3; Matthew 5:14–16</t>
         </is>
       </c>
-      <c r="F27" s="10" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Record it &amp; review it</t>
         </is>
       </c>
-      <c r="G27" s="10" t="inlineStr">
+      <c r="G27" s="9" t="inlineStr">
         <is>
           <t>Run &amp; record the full set; polish</t>
         </is>
       </c>
-      <c r="H27" s="10" t="inlineStr"/>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>Living Hope; Graves Into Gardens; Isn't She Lovely; King of Kings</t>
+        </is>
+      </c>
+      <c r="I27" s="9" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="9" t="inlineStr">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>Sun Feb 21</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>Winter</t>
         </is>
       </c>
-      <c r="D28" s="10" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>The one thing</t>
         </is>
       </c>
-      <c r="E28" s="10" t="inlineStr">
+      <c r="E28" s="9" t="inlineStr">
         <is>
           <t>Psalm 27:4</t>
         </is>
       </c>
-      <c r="F28" s="10" t="inlineStr">
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>Put it together &amp; what's next</t>
         </is>
       </c>
-      <c r="G28" s="10" t="inlineStr">
+      <c r="G28" s="9" t="inlineStr">
         <is>
           <t>Full-set 'final' + next-step conversations</t>
         </is>
       </c>
-      <c r="H28" s="6" t="inlineStr">
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>Living Hope; Graves Into Gardens; Isn't She Lovely; King of Kings</t>
+        </is>
+      </c>
+      <c r="I28" s="9" t="inlineStr">
         <is>
           <t>MILESTONE: full connected set. Plan spring term.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:H28"/>
+  <autoFilter ref="A3:I28"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>